<commit_message>
Update gold data automatically
</commit_message>
<xml_diff>
--- a/data/gold_data.xlsx
+++ b/data/gold_data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1546"/>
+  <dimension ref="A1:I1547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42182,6 +42182,33 @@
       </c>
       <c r="I1546" t="inlineStr"/>
     </row>
+    <row r="1547">
+      <c r="A1547" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B1547" t="n">
+        <v>5128.7998046875</v>
+      </c>
+      <c r="C1547" t="n">
+        <v>5221.89990234375</v>
+      </c>
+      <c r="D1547" t="n">
+        <v>5120.39990234375</v>
+      </c>
+      <c r="E1547" t="n">
+        <v>5205.89990234375</v>
+      </c>
+      <c r="F1547" t="n">
+        <v>85864</v>
+      </c>
+      <c r="G1547" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1547" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1547" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>